<commit_message>
fix: login  page and sheet loading logic
</commit_message>
<xml_diff>
--- a/data/FG Stock as on 31-Jul-26.xlsx
+++ b/data/FG Stock as on 31-Jul-26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/AI Matics/Fibro/ROL Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A7DB2D-6C67-B14D-98AE-60CD67042287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F21C9F51-C920-FC4A-B2A0-78BEDA22F0D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export" sheetId="1" r:id="rId1"/>
@@ -56783,6 +56783,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C3904" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>